<commit_message>
feat: theme bundles from GitHub Pages
- Theme groups and the catalog are remote, loaded from vircatodev.github.io/FivesGame/content/<platform>; previews stay in the player, so the menus work offline
- The loading screen downloads every theme at start; a game started offline downloads a missing theme when a menu opens it, with progress and Retry or Back
- IThemeDownloads over Addressables, ThemeDownloadGate for the menus, LoadingScreen shows again for downloads
- tools/unity.sh: content-build and content (update) build bundles, publish and publish-content deploy the game and the content separately without replacing each other
- FivesGame > Content menu: play mode from the server or the asset database, build content, clear downloaded content
- The gameplay screen smoke test runs without the Boot scene and in asset database mode, whatever this machine uses
- docs/CONTENT.md: how content is built, published and updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Localization/Strings.xlsx
+++ b/Localization/Strings.xlsx
@@ -1,2033 +1,2495 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <sheets>
-    <sheet name="UI" sheetId="1" r:id="rId1"/>
+    <sheet name="UI" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <numFmts count="0"/>
+  <fonts count="3">
     <font>
+      <name val="Calibri"/>
       <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
-      <b/>
+      <name val="Calibri"/>
+      <b val="1"/>
       <sz val="11"/>
+    </font>
+    <font>
       <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf/>
-    <xf fontId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  </cellStyles>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
+</file>
+
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H49"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="40" customWidth="1"/>
-    <col min="3" max="3" width="34" customWidth="1"/>
-    <col min="4" max="4" width="34" customWidth="1"/>
-    <col min="5" max="5" width="34" customWidth="1"/>
-    <col min="6" max="6" width="34" customWidth="1"/>
-    <col min="7" max="7" width="34" customWidth="1"/>
-    <col min="8" max="8" width="34" customWidth="1"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">Key</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">Comment</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">en</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">ru</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">fr</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">it</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">de</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr" s="1">
-        <is>
-          <t xml:space="preserve">es</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Comment</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>ru</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>fr</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>it</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>de</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>es</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">header.settings</t>
+          <t>header.settings</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Header button; draft: FR/IT/DE/ES need a native check</t>
+          <t>Header button; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Settings</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Настройки</t>
+          <t>Настройки</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Réglages</t>
+          <t>Réglages</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Impostazioni</t>
+          <t>Impostazioni</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Einstellungen</t>
+          <t>Einstellungen</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ajustes</t>
+          <t>Ajustes</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">header.back</t>
+          <t>header.back</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Header button; draft: FR/IT/DE/ES need a native check</t>
+          <t>Header button; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Back</t>
+          <t>Back</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Назад</t>
+          <t>Назад</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retour</t>
+          <t>Retour</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Indietro</t>
+          <t>Indietro</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zurück</t>
+          <t>Zurück</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Atrás</t>
+          <t>Atrás</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">settings.title</t>
+          <t>settings.title</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Settings popup title; draft: FR/IT/DE/ES need a native check</t>
+          <t>Settings popup title; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Settings</t>
+          <t>Settings</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Настройки</t>
+          <t>Настройки</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Réglages</t>
+          <t>Réglages</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Impostazioni</t>
+          <t>Impostazioni</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Einstellungen</t>
+          <t>Einstellungen</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ajustes</t>
+          <t>Ajustes</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">common.play</t>
+          <t>common.play</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Main menu button; puzzle card status; draft: FR/IT/DE/ES need a native check</t>
+          <t>Main menu button; puzzle card status; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Play</t>
+          <t>Play</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Играть</t>
+          <t>Играть</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jouer</t>
+          <t>Jouer</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gioca</t>
+          <t>Gioca</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spielen</t>
+          <t>Spielen</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jugar</t>
+          <t>Jugar</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">menu.levels</t>
+          <t>menu.levels</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Main menu button; draft: FR/IT/DE/ES need a native check</t>
+          <t>Main menu button; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Levels</t>
+          <t>Levels</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Уровни</t>
+          <t>Уровни</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Niveaux</t>
+          <t>Niveaux</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Livelli</t>
+          <t>Livelli</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Level</t>
+          <t>Level</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Niveles</t>
+          <t>Niveles</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">select.themes</t>
+          <t>select.themes</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Select screen title; draft: FR/IT/DE/ES need a native check</t>
+          <t>Select screen title; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">SELECT THEME</t>
+          <t>SELECT THEME</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">ВЫБЕРИ ТЕМУ</t>
+          <t>ВЫБЕРИ ТЕМУ</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t xml:space="preserve">CHOISIS UN THÈME</t>
+          <t>CHOISIS UN THÈME</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t xml:space="preserve">SCEGLI UN TEMA</t>
+          <t>SCEGLI UN TEMA</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t xml:space="preserve">WÄHLE EIN THEMA</t>
+          <t>WÄHLE EIN THEMA</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t xml:space="preserve">ELIGE UN TEMA</t>
+          <t>ELIGE UN TEMA</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">select.puzzles</t>
+          <t>select.puzzles</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Select screen title; draft: FR/IT/DE/ES need a native check</t>
+          <t>Select screen title; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">SELECT PUZZLE</t>
+          <t>SELECT PUZZLE</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">ВЫБЕРИ ПАЗЛ</t>
+          <t>ВЫБЕРИ ПАЗЛ</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t xml:space="preserve">CHOISIS UN PUZZLE</t>
+          <t>CHOISIS UN PUZZLE</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t xml:space="preserve">SCEGLI UN PUZZLE</t>
+          <t>SCEGLI UN PUZZLE</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t xml:space="preserve">WÄHLE EIN PUZZLE</t>
+          <t>WÄHLE EIN PUZZLE</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t xml:space="preserve">ELIGE UN PUZZLE</t>
+          <t>ELIGE UN PUZZLE</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">select.sticker</t>
+          <t>select.sticker</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sticker on the select screen; &lt;br&gt; is a line break; draft: FR/IT/DE/ES need a native check</t>
+          <t>Sticker on the select screen; &lt;br&gt; is a line break; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Choose&lt;br&gt;your&lt;br&gt;theme!</t>
+          <t>Choose&lt;br&gt;your&lt;br&gt;theme!</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Выбери&lt;br&gt;свою&lt;br&gt;тему!</t>
+          <t>Выбери&lt;br&gt;свою&lt;br&gt;тему!</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Choisis&lt;br&gt;ton&lt;br&gt;thème !</t>
+          <t>Choisis&lt;br&gt;ton&lt;br&gt;thème !</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scegli&lt;br&gt;il tuo&lt;br&gt;tema!</t>
+          <t>Scegli&lt;br&gt;il tuo&lt;br&gt;tema!</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wähle&lt;br&gt;dein&lt;br&gt;Thema!</t>
+          <t>Wähle&lt;br&gt;dein&lt;br&gt;Thema!</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t xml:space="preserve">¡Elige&lt;br&gt;tu&lt;br&gt;tema!</t>
+          <t>¡Elige&lt;br&gt;tu&lt;br&gt;tema!</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">select.open</t>
+          <t>select.open</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Locked theme; {0} = price in stars; draft: FR/IT/DE/ES need a native check</t>
+          <t>Locked theme; {0} = price in stars; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open {0}</t>
+          <t>Open {0}</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Открыть {0}</t>
+          <t>Открыть {0}</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ouvrir {0}</t>
+          <t>Ouvrir {0}</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Apri {0}</t>
+          <t>Apri {0}</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Öffnen {0}</t>
+          <t>Öffnen {0}</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Abrir {0}</t>
+          <t>Abrir {0}</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">select.theme_completed</t>
+          <t>select.theme_completed</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Theme card when every puzzle is done; draft: FR/IT/DE/ES need a native check</t>
+          <t>Theme card when every puzzle is done; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">COMPLETED</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">ГОТОВО</t>
+          <t>ГОТОВО</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">TERMINÉ</t>
+          <t>TERMINÉ</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t xml:space="preserve">COMPLETATO</t>
+          <t>COMPLETATO</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t xml:space="preserve">GESCHAFFT</t>
+          <t>GESCHAFFT</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t xml:space="preserve">COMPLETADO</t>
+          <t>COMPLETADO</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">select.puzzle_completed</t>
+          <t>select.puzzle_completed</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Puzzle card when done; draft: FR/IT/DE/ES need a native check</t>
+          <t>Puzzle card when done; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Complete</t>
+          <t>Complete</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Собран</t>
+          <t>Собран</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Terminé</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Completato</t>
+          <t>Completato</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fertig</t>
+          <t>Fertig</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Completado</t>
+          <t>Completado</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">game.undo</t>
+          <t>game.undo</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Undo button, keep short; draft: FR/IT/DE/ES need a native check</t>
+          <t>Undo button, keep short; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Undo</t>
+          <t>Undo</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Отмена</t>
+          <t>Отмена</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Annuler</t>
+          <t>Annuler</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Annulla</t>
+          <t>Annulla</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zurück</t>
+          <t>Zurück</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Deshacer</t>
+          <t>Deshacer</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">game.moves</t>
+          <t>game.moves</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">{0} = move count; draft: FR/IT/DE/ES need a native check</t>
+          <t>{0} = move count; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moves: {0}</t>
+          <t>Moves: {0}</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ходы: {0}</t>
+          <t>Ходы: {0}</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Coups : {0}</t>
+          <t>Coups : {0}</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mosse: {0}</t>
+          <t>Mosse: {0}</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Züge: {0}</t>
+          <t>Züge: {0}</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jugadas: {0}</t>
+          <t>Jugadas: {0}</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">result.title</t>
+          <t>result.title</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Result screen title; draft: FR/IT/DE/ES need a native check</t>
+          <t>Result screen title; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Level Complete</t>
+          <t>Level Complete</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Уровень пройден</t>
+          <t>Уровень пройден</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Niveau terminé</t>
+          <t>Niveau terminé</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Livello completato</t>
+          <t>Livello completato</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Level geschafft</t>
+          <t>Level geschafft</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t xml:space="preserve">¡Nivel completado!</t>
+          <t>¡Nivel completado!</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">result.reward</t>
+          <t>result.reward</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Result screen label; draft: FR/IT/DE/ES need a native check</t>
+          <t>Result screen label; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">REWARD</t>
+          <t>REWARD</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">НАГРАДА</t>
+          <t>НАГРАДА</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t xml:space="preserve">RÉCOMPENSE</t>
+          <t>RÉCOMPENSE</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t xml:space="preserve">PREMIO</t>
+          <t>PREMIO</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t xml:space="preserve">BELOHNUNG</t>
+          <t>BELOHNUNG</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t xml:space="preserve">PREMIO</t>
+          <t>PREMIO</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">result.stars</t>
+          <t>result.stars</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">{0} = 10 or 20 stars (RU form fits these numbers); draft: FR/IT/DE/ES need a native check</t>
+          <t>{0} = 10 or 20 stars (RU form fits these numbers); draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">+{0} Stars</t>
+          <t>+{0} Stars</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">+{0} звезд</t>
+          <t>+{0} звезд</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t xml:space="preserve">+{0} étoiles</t>
+          <t>+{0} étoiles</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t xml:space="preserve">+{0} stelle</t>
+          <t>+{0} stelle</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t xml:space="preserve">+{0} Sterne</t>
+          <t>+{0} Sterne</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t xml:space="preserve">+{0} estrellas</t>
+          <t>+{0} estrellas</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">result.stats</t>
+          <t>result.stats</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">{0} = moves, {1} = time mm:ss; draft: FR/IT/DE/ES need a native check</t>
+          <t>{0} = moves, {1} = time mm:ss; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moves: {0}  ·  Time: {1}</t>
+          <t>Moves: {0}  ·  Time: {1}</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ходы: {0}  ·  Время: {1}</t>
+          <t>Ходы: {0}  ·  Время: {1}</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Coups : {0}  ·  Temps : {1}</t>
+          <t>Coups : {0}  ·  Temps : {1}</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mosse: {0}  ·  Tempo: {1}</t>
+          <t>Mosse: {0}  ·  Tempo: {1}</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Züge: {0}  ·  Zeit: {1}</t>
+          <t>Züge: {0}  ·  Zeit: {1}</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jugadas: {0}  ·  Tiempo: {1}</t>
+          <t>Jugadas: {0}  ·  Tiempo: {1}</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">result.claim</t>
+          <t>result.claim</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Result button; draft: FR/IT/DE/ES need a native check</t>
+          <t>Result button; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Claim</t>
+          <t>Claim</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Забрать</t>
+          <t>Забрать</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Récupérer</t>
+          <t>Récupérer</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ritira</t>
+          <t>Ritira</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Abholen</t>
+          <t>Abholen</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recoger</t>
+          <t>Recoger</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">result.claim_double</t>
+          <t>result.claim_double</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Result button, doubled reward; draft: FR/IT/DE/ES need a native check</t>
+          <t>Result button, doubled reward; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t xml:space="preserve">x2 Claim</t>
+          <t>x2 Claim</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Забрать x2</t>
+          <t>Забрать x2</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Récupérer x2</t>
+          <t>Récupérer x2</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ritira x2</t>
+          <t>Ritira x2</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Abholen x2</t>
+          <t>Abholen x2</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recoger x2</t>
+          <t>Recoger x2</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">theme.dogs</t>
+          <t>theme.dogs</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Theme name; draft: FR/IT/DE/ES need a native check</t>
+          <t>Theme name; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dogs</t>
+          <t>Dogs</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Собаки</t>
+          <t>Собаки</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chiens</t>
+          <t>Chiens</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cani</t>
+          <t>Cani</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hunde</t>
+          <t>Hunde</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Perros</t>
+          <t>Perros</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">theme.cats</t>
+          <t>theme.cats</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Theme name; draft: FR/IT/DE/ES need a native check</t>
+          <t>Theme name; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cats</t>
+          <t>Cats</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Кошки</t>
+          <t>Кошки</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chats</t>
+          <t>Chats</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gatti</t>
+          <t>Gatti</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Katzen</t>
+          <t>Katzen</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gatos</t>
+          <t>Gatos</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">theme.pets</t>
+          <t>theme.pets</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Theme name; draft: FR/IT/DE/ES need a native check</t>
+          <t>Theme name; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pets</t>
+          <t>Pets</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Питомцы</t>
+          <t>Питомцы</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Animaux</t>
+          <t>Animaux</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Animali</t>
+          <t>Animali</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Haustiere</t>
+          <t>Haustiere</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mascotas</t>
+          <t>Mascotas</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">puzzle.dogs.corgi</t>
+          <t>puzzle.dogs.corgi</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Puzzle name; draft: FR/IT/DE/ES need a native check</t>
+          <t>Puzzle name; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Corgi</t>
+          <t>Corgi</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Корги</t>
+          <t>Корги</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Corgi</t>
+          <t>Corgi</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Corgi</t>
+          <t>Corgi</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Corgi</t>
+          <t>Corgi</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Corgi</t>
+          <t>Corgi</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">puzzle.dogs.corgi.about</t>
+          <t>puzzle.dogs.corgi.about</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Puzzle description; draft: FR/IT/DE/ES need a native check</t>
+          <t>Puzzle description; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Corgi is a miniature sheepdog, a herding dog that helped Welsh farmers herd sheep.</t>
+          <t>Corgi is a miniature sheepdog, a herding dog that helped Welsh farmers herd sheep.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Корги - маленькая пастушья собака. Она помогала валлийским фермерам пасти овец.</t>
+          <t>Корги - маленькая пастушья собака. Она помогала валлийским фермерам пасти овец.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Le corgi est un petit chien de berger qui aidait les fermiers gallois à garder les moutons.</t>
+          <t>Le corgi est un petit chien de berger qui aidait les fermiers gallois à garder les moutons.</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Il corgi è un piccolo cane da pastore che aiutava i contadini gallesi a guidare le pecore.</t>
+          <t>Il corgi è un piccolo cane da pastore che aiutava i contadini gallesi a guidare le pecore.</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Der Corgi ist ein kleiner Hütehund, der walisischen Bauern beim Schafehüten half.</t>
+          <t>Der Corgi ist ein kleiner Hütehund, der walisischen Bauern beim Schafehüten half.</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t xml:space="preserve">El corgi es un pequeño perro pastor que ayudaba a los granjeros galeses con las ovejas.</t>
+          <t>El corgi es un pequeño perro pastor que ayudaba a los granjeros galeses con las ovejas.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">puzzle.dogs.pug</t>
+          <t>puzzle.dogs.pug</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Puzzle name; draft: FR/IT/DE/ES need a native check</t>
+          <t>Puzzle name; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pug</t>
+          <t>Pug</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Мопс</t>
+          <t>Мопс</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Carlin</t>
+          <t>Carlin</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Carlino</t>
+          <t>Carlino</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mops</t>
+          <t>Mops</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Carlino</t>
+          <t>Carlino</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">puzzle.dogs.pug.about</t>
+          <t>puzzle.dogs.pug.about</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Puzzle description; draft: FR/IT/DE/ES need a native check</t>
+          <t>Puzzle description; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Pug is a stocky, square-bodied dog.</t>
+          <t>The Pug is a stocky, square-bodied dog.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Мопс - крепкая собака с квадратным телом.</t>
+          <t>Мопс - крепкая собака с квадратным телом.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Le carlin est un petit chien trapu et carré.</t>
+          <t>Le carlin est un petit chien trapu et carré.</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Il carlino è un cane robusto dal corpo quadrato.</t>
+          <t>Il carlino è un cane robusto dal corpo quadrato.</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Der Mops ist ein kräftiger Hund mit quadratischem Körper.</t>
+          <t>Der Mops ist ein kräftiger Hund mit quadratischem Körper.</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t xml:space="preserve">El carlino es un perro robusto de cuerpo cuadrado.</t>
+          <t>El carlino es un perro robusto de cuerpo cuadrado.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">puzzle.dogs.shepherd</t>
+          <t>puzzle.dogs.shepherd</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Puzzle name; draft: FR/IT/DE/ES need a native check</t>
+          <t>Puzzle name; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Shepherd</t>
+          <t>Shepherd</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Овчарка</t>
+          <t>Овчарка</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Berger allemand</t>
+          <t>Berger allemand</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pastore tedesco</t>
+          <t>Pastore tedesco</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Schäferhund</t>
+          <t>Schäferhund</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pastor alemán</t>
+          <t>Pastor alemán</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">puzzle.dogs.shepherd.about</t>
+          <t>puzzle.dogs.shepherd.about</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Puzzle description; draft: FR/IT/DE/ES need a native check</t>
+          <t>Puzzle description; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t xml:space="preserve">The German Shepherd is a herding dog known for its courage, loyalty and protective instinct.</t>
+          <t>The German Shepherd is a herding dog known for its courage, loyalty and protective instinct.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Немецкая овчарка - пастушья собака, известная смелостью, верностью и умением защищать.</t>
+          <t>Немецкая овчарка - пастушья собака, известная смелостью, верностью и умением защищать.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Le berger allemand est un chien de berger courageux, fidèle et protecteur.</t>
+          <t>Le berger allemand est un chien de berger courageux, fidèle et protecteur.</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Il pastore tedesco è un cane da pastore coraggioso, fedele e protettivo.</t>
+          <t>Il pastore tedesco è un cane da pastore coraggioso, fedele e protettivo.</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Der Deutsche Schäferhund ist ein mutiger, treuer und beschützender Hütehund.</t>
+          <t>Der Deutsche Schäferhund ist ein mutiger, treuer und beschützender Hütehund.</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t xml:space="preserve">El pastor alemán es un perro pastor valiente, leal y protector.</t>
+          <t>El pastor alemán es un perro pastor valiente, leal y protector.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">puzzle.cats.siamese</t>
+          <t>puzzle.cats.siamese</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Puzzle name; draft: FR/IT/DE/ES need a native check</t>
+          <t>Puzzle name; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Siamese</t>
+          <t>Siamese</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Сиамская</t>
+          <t>Сиамская</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Siamois</t>
+          <t>Siamois</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Siamese</t>
+          <t>Siamese</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Siamkatze</t>
+          <t>Siamkatze</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Siamés</t>
+          <t>Siamés</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">puzzle.cats.siamese.about</t>
+          <t>puzzle.cats.siamese.about</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Puzzle description; draft: FR/IT/DE/ES need a native check</t>
+          <t>Puzzle description; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Siamese cat has bright blue eyes and dark ears, paws and tail.</t>
+          <t>The Siamese cat has bright blue eyes and dark ears, paws and tail.</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t xml:space="preserve">У сиамской кошки ярко-голубые глаза и темные ушки, лапки и хвост.</t>
+          <t>У сиамской кошки ярко-голубые глаза и темные ушки, лапки и хвост.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Le chat siamois a des yeux bleu vif et des oreilles, des pattes et une queue foncées.</t>
+          <t>Le chat siamois a des yeux bleu vif et des oreilles, des pattes et une queue foncées.</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Il gatto siamese ha occhi azzurri brillanti e orecchie, zampe e coda scure.</t>
+          <t>Il gatto siamese ha occhi azzurri brillanti e orecchie, zampe e coda scure.</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Die Siamkatze hat leuchtend blaue Augen und dunkle Ohren, Pfoten und einen dunklen Schwanz.</t>
+          <t>Die Siamkatze hat leuchtend blaue Augen und dunkle Ohren, Pfoten und einen dunklen Schwanz.</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t xml:space="preserve">El gato siamés tiene ojos azules brillantes y orejas, patas y cola oscuras.</t>
+          <t>El gato siamés tiene ojos azules brillantes y orejas, patas y cola oscuras.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">puzzle.cats.british</t>
+          <t>puzzle.cats.british</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Puzzle name; draft: FR/IT/DE/ES need a native check</t>
+          <t>Puzzle name; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t xml:space="preserve">British</t>
+          <t>British</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Британская</t>
+          <t>Британская</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t xml:space="preserve">British</t>
+          <t>British</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t xml:space="preserve">British</t>
+          <t>British</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Britisch Kurzhaar</t>
+          <t>Britisch Kurzhaar</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Británico</t>
+          <t>Británico</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">puzzle.cats.british.about</t>
+          <t>puzzle.cats.british.about</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Puzzle description; draft: FR/IT/DE/ES need a native check</t>
+          <t>Puzzle description; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t xml:space="preserve">The British Shorthair is a calm, cuddly cat with thick grey fur.</t>
+          <t>The British Shorthair is a calm, cuddly cat with thick grey fur.</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Британская короткошерстная - спокойная и ласковая кошка с густой серой шерстью.</t>
+          <t>Британская короткошерстная - спокойная и ласковая кошка с густой серой шерстью.</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Le British Shorthair est un chat calme et câlin au pelage gris épais.</t>
+          <t>Le British Shorthair est un chat calme et câlin au pelage gris épais.</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Il British Shorthair è un gatto calmo e coccolone dal folto pelo grigio.</t>
+          <t>Il British Shorthair è un gatto calmo e coccolone dal folto pelo grigio.</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Die Britisch Kurzhaar ist eine ruhige, verschmuste Katze mit dichtem grauem Fell.</t>
+          <t>Die Britisch Kurzhaar ist eine ruhige, verschmuste Katze mit dichtem grauem Fell.</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t xml:space="preserve">El británico de pelo corto es un gato tranquilo y mimoso con un pelaje gris espeso.</t>
+          <t>El británico de pelo corto es un gato tranquilo y mimoso con un pelaje gris espeso.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">puzzle.cats.ginger</t>
+          <t>puzzle.cats.ginger</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Puzzle name; draft: FR/IT/DE/ES need a native check</t>
+          <t>Puzzle name; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ginger</t>
+          <t>Ginger</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Рыжий</t>
+          <t>Рыжий</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Roux</t>
+          <t>Roux</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rosso</t>
+          <t>Rosso</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rote Katze</t>
+          <t>Rote Katze</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pelirrojo</t>
+          <t>Pelirrojo</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">puzzle.cats.ginger.about</t>
+          <t>puzzle.cats.ginger.about</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Puzzle description; draft: FR/IT/DE/ES need a native check</t>
+          <t>Puzzle description; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ginger cats have warm orange fur with stripes and love to play.</t>
+          <t>Ginger cats have warm orange fur with stripes and love to play.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t xml:space="preserve">У рыжих котов теплая оранжевая шерсть в полоску, и они обожают играть.</t>
+          <t>У рыжих котов теплая оранжевая шерсть в полоску, и они обожают играть.</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Les chats roux ont un pelage orange rayé et adorent jouer.</t>
+          <t>Les chats roux ont un pelage orange rayé et adorent jouer.</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t xml:space="preserve">I gatti rossi hanno un caldo pelo arancione a strisce e adorano giocare.</t>
+          <t>I gatti rossi hanno un caldo pelo arancione a strisce e adorano giocare.</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rote Katzen haben warmes, gestreiftes orangefarbenes Fell und spielen gern.</t>
+          <t>Rote Katzen haben warmes, gestreiftes orangefarbenes Fell und spielen gern.</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Los gatos pelirrojos tienen un cálido pelaje naranja a rayas y les encanta jugar.</t>
+          <t>Los gatos pelirrojos tienen un cálido pelaje naranja a rayas y les encanta jugar.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">puzzle.pets.biscuit</t>
+          <t>puzzle.pets.biscuit</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pet name; draft: FR/IT/DE/ES need a native check</t>
+          <t>Pet name; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Biscuit</t>
+          <t>Biscuit</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Бисквит</t>
+          <t>Бисквит</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Biscuit</t>
+          <t>Biscuit</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Biscuit</t>
+          <t>Biscuit</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Biscuit</t>
+          <t>Biscuit</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Biscuit</t>
+          <t>Biscuit</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">puzzle.pets.biscuit.about</t>
+          <t>puzzle.pets.biscuit.about</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Puzzle description; draft: FR/IT/DE/ES need a native check</t>
+          <t>Puzzle description; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Biscuit is a happy Corgi who loves long walks and belly rubs.</t>
+          <t>Biscuit is a happy Corgi who loves long walks and belly rubs.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Бисквит - веселый корги, который обожает долгие прогулки и когда ему чешут животик.</t>
+          <t>Бисквит - веселый корги, который обожает долгие прогулки и когда ему чешут животик.</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Biscuit est un corgi joyeux qui adore les longues promenades et les câlins sur le ventre.</t>
+          <t>Biscuit est un corgi joyeux qui adore les longues promenades et les câlins sur le ventre.</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Biscuit è un corgi allegro che adora le lunghe passeggiate e le grattatine sulla pancia.</t>
+          <t>Biscuit è un corgi allegro che adora le lunghe passeggiate e le grattatine sulla pancia.</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Biscuit ist ein fröhlicher Corgi, der lange Spaziergänge und Bauchkraulen liebt.</t>
+          <t>Biscuit ist ein fröhlicher Corgi, der lange Spaziergänge und Bauchkraulen liebt.</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Biscuit es un corgi feliz al que le encantan los paseos largos y las caricias en la barriga.</t>
+          <t>Biscuit es un corgi feliz al que le encantan los paseos largos y las caricias en la barriga.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">puzzle.pets.luna</t>
+          <t>puzzle.pets.luna</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pet name; draft: FR/IT/DE/ES need a native check</t>
+          <t>Pet name; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Luna</t>
+          <t>Luna</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Луна</t>
+          <t>Луна</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Luna</t>
+          <t>Luna</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Luna</t>
+          <t>Luna</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Luna</t>
+          <t>Luna</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Luna</t>
+          <t>Luna</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">puzzle.pets.luna.about</t>
+          <t>puzzle.pets.luna.about</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Puzzle description; draft: FR/IT/DE/ES need a native check</t>
+          <t>Puzzle description; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Luna is a curious Siamese kitten with sky-blue eyes.</t>
+          <t>Luna is a curious Siamese kitten with sky-blue eyes.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Луна - любопытный сиамский котенок с небесно-голубыми глазами.</t>
+          <t>Луна - любопытный сиамский котенок с небесно-голубыми глазами.</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Luna est une chatonne siamoise curieuse aux yeux bleu ciel.</t>
+          <t>Luna est une chatonne siamoise curieuse aux yeux bleu ciel.</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Luna è una gattina siamese curiosa con gli occhi azzurro cielo.</t>
+          <t>Luna è una gattina siamese curiosa con gli occhi azzurro cielo.</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Luna ist ein neugieriges Siamkätzchen mit himmelblauen Augen.</t>
+          <t>Luna ist ein neugieriges Siamkätzchen mit himmelblauen Augen.</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Luna es una gatita siamesa curiosa de ojos azul cielo.</t>
+          <t>Luna es una gatita siamesa curiosa de ojos azul cielo.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">puzzle.pets.muffin</t>
+          <t>puzzle.pets.muffin</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pet name; draft: FR/IT/DE/ES need a native check</t>
+          <t>Pet name; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Muffin</t>
+          <t>Muffin</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Маффин</t>
+          <t>Маффин</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Muffin</t>
+          <t>Muffin</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Muffin</t>
+          <t>Muffin</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Muffin</t>
+          <t>Muffin</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Muffin</t>
+          <t>Muffin</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">puzzle.pets.muffin.about</t>
+          <t>puzzle.pets.muffin.about</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Puzzle description; draft: FR/IT/DE/ES need a native check</t>
+          <t>Puzzle description; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Muffin is a cheeky Pug who snores when she sleeps.</t>
+          <t>Muffin is a cheeky Pug who snores when she sleeps.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Маффин - озорная мопсиха, которая храпит во сне.</t>
+          <t>Маффин - озорная мопсиха, которая храпит во сне.</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Muffin est une petite carline espiègle qui ronfle en dormant.</t>
+          <t>Muffin est une petite carline espiègle qui ronfle en dormant.</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Muffin è una carlina birichina che russa quando dorme.</t>
+          <t>Muffin è una carlina birichina che russa quando dorme.</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Muffin ist eine freche Mopsdame, die im Schlaf schnarcht.</t>
+          <t>Muffin ist eine freche Mopsdame, die im Schlaf schnarcht.</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Muffin es una carlina traviesa que ronca cuando duerme.</t>
+          <t>Muffin es una carlina traviesa que ronca cuando duerme.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">puzzle.pets.smokey</t>
+          <t>puzzle.pets.smokey</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pet name; draft: FR/IT/DE/ES need a native check</t>
+          <t>Pet name; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smokey</t>
+          <t>Smokey</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Дымок</t>
+          <t>Дымок</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smokey</t>
+          <t>Smokey</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smokey</t>
+          <t>Smokey</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smokey</t>
+          <t>Smokey</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smokey</t>
+          <t>Smokey</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">puzzle.pets.smokey.about</t>
+          <t>puzzle.pets.smokey.about</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Puzzle description; draft: FR/IT/DE/ES need a native check</t>
+          <t>Puzzle description; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smokey is a fluffy grey cat who loves a warm sunny spot.</t>
+          <t>Smokey is a fluffy grey cat who loves a warm sunny spot.</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Дымок - пушистый серый кот, который любит теплое солнечное местечко.</t>
+          <t>Дымок - пушистый серый кот, который любит теплое солнечное местечко.</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smokey est un chat gris tout doux qui adore les coins chauds et ensoleillés.</t>
+          <t>Smokey est un chat gris tout doux qui adore les coins chauds et ensoleillés.</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smokey è un soffice gatto grigio che ama gli angolini caldi e soleggiati.</t>
+          <t>Smokey è un soffice gatto grigio che ama gli angolini caldi e soleggiati.</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smokey ist ein flauschiger grauer Kater, der warme Sonnenplätze liebt.</t>
+          <t>Smokey ist ein flauschiger grauer Kater, der warme Sonnenplätze liebt.</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smokey es un gato gris y esponjoso al que le encantan los rincones cálidos y soleados.</t>
+          <t>Smokey es un gato gris y esponjoso al que le encantan los rincones cálidos y soleados.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">puzzle.pets.rex</t>
+          <t>puzzle.pets.rex</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pet name; draft: FR/IT/DE/ES need a native check</t>
+          <t>Pet name; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rex</t>
+          <t>Rex</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Рекс</t>
+          <t>Рекс</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rex</t>
+          <t>Rex</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rex</t>
+          <t>Rex</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rex</t>
+          <t>Rex</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rex</t>
+          <t>Rex</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">puzzle.pets.rex.about</t>
+          <t>puzzle.pets.rex.about</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Puzzle description; draft: FR/IT/DE/ES need a native check</t>
+          <t>Puzzle description; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rex is a brave Shepherd who always guards the garden.</t>
+          <t>Rex is a brave Shepherd who always guards the garden.</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Рекс - смелая овчарка, которая всегда охраняет сад.</t>
+          <t>Рекс - смелая овчарка, которая всегда охраняет сад.</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rex est un berger courageux qui garde toujours le jardin.</t>
+          <t>Rex est un berger courageux qui garde toujours le jardin.</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rex è un pastore coraggioso che fa sempre la guardia al giardino.</t>
+          <t>Rex è un pastore coraggioso che fa sempre la guardia al giardino.</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rex ist ein mutiger Schäferhund, der immer den Garten bewacht.</t>
+          <t>Rex ist ein mutiger Schäferhund, der immer den Garten bewacht.</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rex es un pastor valiente que siempre vigila el jardín.</t>
+          <t>Rex es un pastor valiente que siempre vigila el jardín.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">puzzle.pets.tiger</t>
+          <t>puzzle.pets.tiger</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pet name; draft: FR/IT/DE/ES need a native check</t>
+          <t>Pet name; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tiger</t>
+          <t>Tiger</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Тигр</t>
+          <t>Тигр</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tigre</t>
+          <t>Tigre</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tigre</t>
+          <t>Tigre</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tiger</t>
+          <t>Tiger</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tigre</t>
+          <t>Tigre</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">puzzle.pets.tiger.about</t>
+          <t>puzzle.pets.tiger.about</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Puzzle description; draft: FR/IT/DE/ES need a native check</t>
+          <t>Puzzle description; draft: FR/IT/DE/ES need a native check</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tiger is a playful ginger kitten who chases butterflies.</t>
+          <t>Tiger is a playful ginger kitten who chases butterflies.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Тигр - игривый рыжий котенок, который гоняется за бабочками.</t>
+          <t>Тигр - игривый рыжий котенок, который гоняется за бабочками.</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tigre est un chaton roux joueur qui court après les papillons.</t>
+          <t>Tigre est un chaton roux joueur qui court après les papillons.</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tigre è un gattino rosso giocherellone che insegue le farfalle.</t>
+          <t>Tigre è un gattino rosso giocherellone che insegue le farfalle.</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tiger ist ein verspieltes rotes Kätzchen, das Schmetterlingen nachjagt.</t>
+          <t>Tiger ist ein verspieltes rotes Kätzchen, das Schmetterlingen nachjagt.</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tigre es un gatito pelirrojo juguetón que persigue mariposas.</t>
+          <t>Tigre es un gatito pelirrojo juguetón que persigue mariposas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>content.offline</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Loading screen when a theme cannot be downloaded; draft: FR/IT/DE/ES need a native check</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>No internet connection. Connect to download this theme.</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Нет подключения к интернету. Подключись, чтобы скачать эту тему.</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Pas de connexion Internet. Connecte-toi pour télécharger ce thème.</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Nessuna connessione a Internet. Connettiti per scaricare questo tema.</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Keine Internetverbindung. Verbinde dich, um dieses Thema herunterzuladen.</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Sin conexión a Internet. Conéctate para descargar este tema.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>common.retry</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Loading screen button after a failed download; draft: FR/IT/DE/ES need a native check</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Retry</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Повторить</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Réessayer</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Riprova</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Nochmal</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Reintentar</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>